<commit_message>
Update schematic, BOM and add 3d models
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nerd Projects\DivergenceMeter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B0E3D81-5E46-4B12-97CC-68BADE9D26B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{830D29D2-CF3F-43E3-95BD-4F14351E0F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Item</t>
   </si>
@@ -48,13 +48,46 @@
     <t>24k ohm resistors</t>
   </si>
   <si>
-    <t>https://www.amazon.com/Voltage-Converter-Supply-10V-13VDC-130V-190V/dp/B0D3766FF3#averageCustomerReviewsAnchor</t>
-  </si>
-  <si>
     <t>https://www.ebay.com/itm/168054788004</t>
   </si>
   <si>
     <t>https://www.ebay.com/itm/332803698406</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>12v wall adapter</t>
+  </si>
+  <si>
+    <t>5.2mm barrel jack female adapter</t>
+  </si>
+  <si>
+    <t>couple cents</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B0BZS6BY6P?smid=A2BHW94NEQUDXN&amp;psc=1</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B0D3766FF3?smid=A3SHE1R0JE35U2&amp;psc=1</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B0B6ZRMQLW?smid=AGOSLUO29ZUJ2&amp;psc=1</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B0DK2THZ85?smid=AT3HD2I36TXBB&amp;psc=1</t>
+  </si>
+  <si>
+    <t>Silver PLA filament</t>
+  </si>
+  <si>
+    <t>Beige PLA filament</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/ELEGOO-Filament-Dimensional-Accuracy-Cardboard/dp/B0CB4935HJ?th=1</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B0B5ZLFTRN?ref=ppx_yo2ov_dt_b_fed_asin_title</t>
   </si>
 </sst>
 </file>
@@ -383,11 +416,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="117.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -416,7 +450,7 @@
         <v>99.95</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -426,6 +460,9 @@
       <c r="B3" t="s">
         <v>6</v>
       </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -438,11 +475,22 @@
         <v>41.94</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="1"/>
+      <c r="C5">
+        <v>5.99</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -455,13 +503,73 @@
         <v>15.99</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>9.99</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>9.99</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>17.09</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10">
+        <v>18.989999999999998</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D6" r:id="rId1" location="averageCustomerReviewsAnchor" xr:uid="{501FEE88-E5F0-4B19-934E-5DB9DB5A5B32}"/>
-    <hyperlink ref="D2" r:id="rId2" xr:uid="{B399A220-4761-4D82-9697-822B9ACBD5FB}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{B399A220-4761-4D82-9697-822B9ACBD5FB}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{A36A11AC-BE45-433B-AE53-82D3A38E15B9}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{9FCAD389-E00A-4D91-87DD-32DD2C9BC445}"/>
+    <hyperlink ref="D8" r:id="rId4" xr:uid="{22199D78-E82D-4F81-B085-4452A22B6F6B}"/>
+    <hyperlink ref="D10" r:id="rId5" xr:uid="{C9C2C497-B5E2-4F4D-BDC8-6A8A9A0DCA2A}"/>
+    <hyperlink ref="D9" r:id="rId6" xr:uid="{2D6CFBF2-6D22-4953-A224-42CDBEF9A2D2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>